<commit_message>
Rebuild combined supply-use tables to proper SEEA EA Table 7.1 format
Replaced the simplified side-by-side combined table with the proper
SEEA EA format (Table 7.1a supply + Table 7.1b use):

Both tables share the same columns:
  Left: Economic units (Fisheries, Tourism, Other, Households, Govt, Global)
  Right: Ecosystem types (Coral reefs M1.3, Seagrass M1.1, Mangroves MFT1.2)
  Far right: TOTAL

Supply table (7.1a): ecosystem columns populated (ecosystems supply services)
Use table (7.1b): economic unit columns populated (sectors use services)
Accounting identity: Total supply = Total use per service row

Category sub-headers: Provisioning (6.1), Regulating (6.2-6.5), Cultural (6.6)
Green headers for supply, teal for use (visual distinction)
Carbon sequestration allocated to Global/Exports column

Updated in: example Excel, template Excel, exercise Excel,
example Word doc, and all print notebook copies.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/s-s-event-bogor/print-notebooks/03-services/10-template.xlsx
+++ b/s-s-event-bogor/print-notebooks/03-services/10-template.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,8 +95,44 @@
       <color rgb="00717171"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00404040"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -127,8 +163,20 @@
         <bgColor rgb="002C745B"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5E8D4"/>
+        <bgColor rgb="00D5E8D4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B2D8D8"/>
+        <bgColor rgb="00B2D8D8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -150,11 +198,55 @@
         <color rgb="00404040"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00404040"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00404040"/>
+      </right>
+      <top style="thin">
+        <color rgb="00404040"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00404040"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00404040"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00404040"/>
+      </right>
+      <top style="thin">
+        <color rgb="00404040"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00404040"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -216,6 +308,50 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2244,485 +2380,662 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Combined Physical Supply and Use Table</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="21" t="n"/>
-      <c r="B2" s="21" t="n"/>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>SUPPLY (by ecosystem)</t>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>SUPPLY TABLE (Table 7.1a)</t>
+        </is>
+      </c>
+      <c r="B1" s="30" t="n"/>
+      <c r="C1" s="30" t="n"/>
+      <c r="D1" s="30" t="n"/>
+      <c r="E1" s="30" t="n"/>
+      <c r="F1" s="30" t="n"/>
+      <c r="G1" s="30" t="n"/>
+      <c r="H1" s="30" t="n"/>
+      <c r="I1" s="30" t="n"/>
+      <c r="J1" s="30" t="n"/>
+      <c r="K1" s="30" t="n"/>
+      <c r="L1" s="30" t="n"/>
+      <c r="M1" s="30" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="22" t="n"/>
+      <c r="B2" s="22" t="n"/>
+      <c r="C2" s="31" t="inlineStr">
+        <is>
+          <t>Economic units</t>
         </is>
       </c>
       <c r="D2" s="22" t="n"/>
       <c r="E2" s="22" t="n"/>
       <c r="F2" s="22" t="n"/>
-      <c r="G2" s="23" t="inlineStr">
-        <is>
-          <t>USE (by beneficiary)</t>
-        </is>
-      </c>
-      <c r="H2" s="21" t="n"/>
-      <c r="I2" s="21" t="n"/>
-      <c r="J2" s="21" t="n"/>
-      <c r="K2" s="21" t="n"/>
-      <c r="L2" s="21" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="G2" s="22" t="n"/>
+      <c r="H2" s="22" t="n"/>
+      <c r="I2" s="31" t="inlineStr">
+        <is>
+          <t>Ecosystem types</t>
+        </is>
+      </c>
+      <c r="J2" s="22" t="n"/>
+      <c r="K2" s="22" t="n"/>
+      <c r="L2" s="22" t="n"/>
+      <c r="M2" s="22" t="n"/>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="32" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="C3" s="25" t="inlineStr">
-        <is>
-          <t>Coral reefs</t>
-        </is>
-      </c>
-      <c r="D3" s="25" t="inlineStr">
-        <is>
-          <t>Seagrass</t>
-        </is>
-      </c>
-      <c r="E3" s="25" t="inlineStr">
-        <is>
-          <t>Mangroves</t>
-        </is>
-      </c>
-      <c r="F3" s="25" t="inlineStr">
-        <is>
-          <t>Total supply</t>
-        </is>
-      </c>
-      <c r="G3" s="26" t="inlineStr">
+      <c r="C3" s="32" t="inlineStr">
         <is>
           <t>Fisheries</t>
         </is>
       </c>
-      <c r="H3" s="26" t="inlineStr">
+      <c r="D3" s="32" t="inlineStr">
         <is>
           <t>Tourism</t>
         </is>
       </c>
-      <c r="I3" s="26" t="inlineStr">
-        <is>
-          <t>Coastal HH</t>
-        </is>
-      </c>
-      <c r="J3" s="26" t="inlineStr">
+      <c r="E3" s="32" t="inlineStr">
+        <is>
+          <t>Other industry</t>
+        </is>
+      </c>
+      <c r="F3" s="32" t="inlineStr">
+        <is>
+          <t>Households</t>
+        </is>
+      </c>
+      <c r="G3" s="32" t="inlineStr">
         <is>
           <t>Govt</t>
         </is>
       </c>
-      <c r="K3" s="26" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="L3" s="26" t="inlineStr">
-        <is>
-          <t>Total use</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="H3" s="32" t="inlineStr">
+        <is>
+          <t>Global/Exports</t>
+        </is>
+      </c>
+      <c r="I3" s="32" t="inlineStr">
+        <is>
+          <t>Coral reefs
+(M1.3)</t>
+        </is>
+      </c>
+      <c r="J3" s="32" t="inlineStr">
+        <is>
+          <t>Seagrass meadows
+(M1.1)</t>
+        </is>
+      </c>
+      <c r="K3" s="32" t="inlineStr">
+        <is>
+          <t>Mangroves
+(MFT1.2)</t>
+        </is>
+      </c>
+      <c r="L3" s="32" t="inlineStr">
+        <is>
+          <t>Total ecosystem</t>
+        </is>
+      </c>
+      <c r="M3" s="32" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="33" t="inlineStr">
+        <is>
+          <t>Provisioning services (SEEA EA 6.1)</t>
+        </is>
+      </c>
+      <c r="B4" s="34" t="n"/>
+      <c r="C4" s="34" t="n"/>
+      <c r="D4" s="34" t="n"/>
+      <c r="E4" s="34" t="n"/>
+      <c r="F4" s="34" t="n"/>
+      <c r="G4" s="34" t="n"/>
+      <c r="H4" s="34" t="n"/>
+      <c r="I4" s="34" t="n"/>
+      <c r="J4" s="34" t="n"/>
+      <c r="K4" s="34" t="n"/>
+      <c r="L4" s="34" t="n"/>
+      <c r="M4" s="34" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="35" t="inlineStr">
         <is>
           <t>Fish provisioning</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B5" s="36" t="inlineStr">
         <is>
           <t>kg/yr</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="7" t="n"/>
-      <c r="H4" s="7" t="n"/>
-      <c r="I4" s="7" t="n"/>
-      <c r="J4" s="7" t="n"/>
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="C5" s="37" t="n"/>
+      <c r="D5" s="37" t="n"/>
+      <c r="E5" s="37" t="n"/>
+      <c r="F5" s="37" t="n"/>
+      <c r="G5" s="37" t="n"/>
+      <c r="H5" s="37" t="n"/>
+      <c r="I5" s="38" t="n"/>
+      <c r="J5" s="38" t="n"/>
+      <c r="K5" s="38" t="n"/>
+      <c r="L5" s="38" t="n"/>
+      <c r="M5" s="38" t="n"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>Regulating &amp; maintenance services (SEEA EA 6.2-6.5)</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="n"/>
+      <c r="C6" s="34" t="n"/>
+      <c r="D6" s="34" t="n"/>
+      <c r="E6" s="34" t="n"/>
+      <c r="F6" s="34" t="n"/>
+      <c r="G6" s="34" t="n"/>
+      <c r="H6" s="34" t="n"/>
+      <c r="I6" s="34" t="n"/>
+      <c r="J6" s="34" t="n"/>
+      <c r="K6" s="34" t="n"/>
+      <c r="L6" s="34" t="n"/>
+      <c r="M6" s="34" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="35" t="inlineStr">
         <is>
           <t>Carbon sequestration</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>Mg CO2/yr</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="B7" s="36" t="inlineStr">
+        <is>
+          <t>Mg CO₂/yr</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="n"/>
+      <c r="D7" s="37" t="n"/>
+      <c r="E7" s="37" t="n"/>
+      <c r="F7" s="37" t="n"/>
+      <c r="G7" s="37" t="n"/>
+      <c r="H7" s="37" t="n"/>
+      <c r="I7" s="38" t="n"/>
+      <c r="J7" s="38" t="n"/>
+      <c r="K7" s="38" t="n"/>
+      <c r="L7" s="38" t="n"/>
+      <c r="M7" s="38" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="35" t="inlineStr">
         <is>
           <t>Coastal protection</t>
         </is>
       </c>
-      <c r="B6" s="27" t="inlineStr">
-        <is>
-          <t>m coastline</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Nursery habitat</t>
-        </is>
-      </c>
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B8" s="36" t="inlineStr">
+        <is>
+          <t>m of coastline</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="n"/>
+      <c r="D8" s="37" t="n"/>
+      <c r="E8" s="37" t="n"/>
+      <c r="F8" s="37" t="n"/>
+      <c r="G8" s="37" t="n"/>
+      <c r="H8" s="37" t="n"/>
+      <c r="I8" s="38" t="n"/>
+      <c r="J8" s="38" t="n"/>
+      <c r="K8" s="38" t="n"/>
+      <c r="L8" s="38" t="n"/>
+      <c r="M8" s="38" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>Nursery habitat support</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="inlineStr">
+        <is>
+          <t>kg fish/yr</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="n"/>
+      <c r="D9" s="37" t="n"/>
+      <c r="E9" s="37" t="n"/>
+      <c r="F9" s="37" t="n"/>
+      <c r="G9" s="37" t="n"/>
+      <c r="H9" s="37" t="n"/>
+      <c r="I9" s="38" t="n"/>
+      <c r="J9" s="38" t="n"/>
+      <c r="K9" s="38" t="n"/>
+      <c r="L9" s="38" t="n"/>
+      <c r="M9" s="38" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>Cultural services (SEEA EA 6.6)</t>
+        </is>
+      </c>
+      <c r="B10" s="34" t="n"/>
+      <c r="C10" s="34" t="n"/>
+      <c r="D10" s="34" t="n"/>
+      <c r="E10" s="34" t="n"/>
+      <c r="F10" s="34" t="n"/>
+      <c r="G10" s="34" t="n"/>
+      <c r="H10" s="34" t="n"/>
+      <c r="I10" s="34" t="n"/>
+      <c r="J10" s="34" t="n"/>
+      <c r="K10" s="34" t="n"/>
+      <c r="L10" s="34" t="n"/>
+      <c r="M10" s="34" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>Recreation &amp; tourism</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="inlineStr">
+        <is>
+          <t>visitors/yr</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="n"/>
+      <c r="D11" s="37" t="n"/>
+      <c r="E11" s="37" t="n"/>
+      <c r="F11" s="37" t="n"/>
+      <c r="G11" s="37" t="n"/>
+      <c r="H11" s="37" t="n"/>
+      <c r="I11" s="38" t="n"/>
+      <c r="J11" s="38" t="n"/>
+      <c r="K11" s="38" t="n"/>
+      <c r="L11" s="38" t="n"/>
+      <c r="M11" s="38" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>Gleaning (subsistence harvest)</t>
+        </is>
+      </c>
+      <c r="B12" s="36" t="inlineStr">
+        <is>
+          <t>hours/yr</t>
+        </is>
+      </c>
+      <c r="C12" s="37" t="n"/>
+      <c r="D12" s="37" t="n"/>
+      <c r="E12" s="37" t="n"/>
+      <c r="F12" s="37" t="n"/>
+      <c r="G12" s="37" t="n"/>
+      <c r="H12" s="37" t="n"/>
+      <c r="I12" s="38" t="n"/>
+      <c r="J12" s="38" t="n"/>
+      <c r="K12" s="38" t="n"/>
+      <c r="L12" s="38" t="n"/>
+      <c r="M12" s="38" t="n"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="39" t="inlineStr">
+        <is>
+          <t>USE TABLE (Table 7.1b)</t>
+        </is>
+      </c>
+      <c r="B14" s="40" t="n"/>
+      <c r="C14" s="40" t="n"/>
+      <c r="D14" s="40" t="n"/>
+      <c r="E14" s="40" t="n"/>
+      <c r="F14" s="40" t="n"/>
+      <c r="G14" s="40" t="n"/>
+      <c r="H14" s="40" t="n"/>
+      <c r="I14" s="40" t="n"/>
+      <c r="J14" s="40" t="n"/>
+      <c r="K14" s="40" t="n"/>
+      <c r="L14" s="40" t="n"/>
+      <c r="M14" s="40" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="41" t="n"/>
+      <c r="B15" s="41" t="n"/>
+      <c r="C15" s="42" t="inlineStr">
+        <is>
+          <t>Economic units</t>
+        </is>
+      </c>
+      <c r="D15" s="41" t="n"/>
+      <c r="E15" s="41" t="n"/>
+      <c r="F15" s="41" t="n"/>
+      <c r="G15" s="41" t="n"/>
+      <c r="H15" s="41" t="n"/>
+      <c r="I15" s="42" t="inlineStr">
+        <is>
+          <t>Ecosystem types</t>
+        </is>
+      </c>
+      <c r="J15" s="41" t="n"/>
+      <c r="K15" s="41" t="n"/>
+      <c r="L15" s="41" t="n"/>
+      <c r="M15" s="41" t="n"/>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="B16" s="43" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>Fisheries</t>
+        </is>
+      </c>
+      <c r="D16" s="43" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="E16" s="43" t="inlineStr">
+        <is>
+          <t>Other industry</t>
+        </is>
+      </c>
+      <c r="F16" s="43" t="inlineStr">
+        <is>
+          <t>Households</t>
+        </is>
+      </c>
+      <c r="G16" s="43" t="inlineStr">
+        <is>
+          <t>Govt</t>
+        </is>
+      </c>
+      <c r="H16" s="43" t="inlineStr">
+        <is>
+          <t>Global/Exports</t>
+        </is>
+      </c>
+      <c r="I16" s="43" t="inlineStr">
+        <is>
+          <t>Coral reefs
+(M1.3)</t>
+        </is>
+      </c>
+      <c r="J16" s="43" t="inlineStr">
+        <is>
+          <t>Seagrass meadows
+(M1.1)</t>
+        </is>
+      </c>
+      <c r="K16" s="43" t="inlineStr">
+        <is>
+          <t>Mangroves
+(MFT1.2)</t>
+        </is>
+      </c>
+      <c r="L16" s="43" t="inlineStr">
+        <is>
+          <t>Total ecosystem</t>
+        </is>
+      </c>
+      <c r="M16" s="43" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="44" t="inlineStr">
+        <is>
+          <t>Provisioning services (SEEA EA 6.1)</t>
+        </is>
+      </c>
+      <c r="B17" s="45" t="n"/>
+      <c r="C17" s="45" t="n"/>
+      <c r="D17" s="45" t="n"/>
+      <c r="E17" s="45" t="n"/>
+      <c r="F17" s="45" t="n"/>
+      <c r="G17" s="45" t="n"/>
+      <c r="H17" s="45" t="n"/>
+      <c r="I17" s="45" t="n"/>
+      <c r="J17" s="45" t="n"/>
+      <c r="K17" s="45" t="n"/>
+      <c r="L17" s="45" t="n"/>
+      <c r="M17" s="45" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>Fish provisioning</t>
+        </is>
+      </c>
+      <c r="B18" s="36" t="inlineStr">
         <is>
           <t>kg/yr</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Recreation</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="C18" s="38" t="n"/>
+      <c r="D18" s="38" t="n"/>
+      <c r="E18" s="38" t="n"/>
+      <c r="F18" s="38" t="n"/>
+      <c r="G18" s="38" t="n"/>
+      <c r="H18" s="38" t="n"/>
+      <c r="I18" s="37" t="n"/>
+      <c r="J18" s="37" t="n"/>
+      <c r="K18" s="37" t="n"/>
+      <c r="L18" s="38" t="n"/>
+      <c r="M18" s="38" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="44" t="inlineStr">
+        <is>
+          <t>Regulating &amp; maintenance services (SEEA EA 6.2-6.5)</t>
+        </is>
+      </c>
+      <c r="B19" s="45" t="n"/>
+      <c r="C19" s="45" t="n"/>
+      <c r="D19" s="45" t="n"/>
+      <c r="E19" s="45" t="n"/>
+      <c r="F19" s="45" t="n"/>
+      <c r="G19" s="45" t="n"/>
+      <c r="H19" s="45" t="n"/>
+      <c r="I19" s="45" t="n"/>
+      <c r="J19" s="45" t="n"/>
+      <c r="K19" s="45" t="n"/>
+      <c r="L19" s="45" t="n"/>
+      <c r="M19" s="45" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>Carbon sequestration</t>
+        </is>
+      </c>
+      <c r="B20" s="36" t="inlineStr">
+        <is>
+          <t>Mg CO₂/yr</t>
+        </is>
+      </c>
+      <c r="C20" s="38" t="n"/>
+      <c r="D20" s="38" t="n"/>
+      <c r="E20" s="38" t="n"/>
+      <c r="F20" s="38" t="n"/>
+      <c r="G20" s="38" t="n"/>
+      <c r="H20" s="38" t="n"/>
+      <c r="I20" s="37" t="n"/>
+      <c r="J20" s="37" t="n"/>
+      <c r="K20" s="37" t="n"/>
+      <c r="L20" s="38" t="n"/>
+      <c r="M20" s="38" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="35" t="inlineStr">
+        <is>
+          <t>Coastal protection</t>
+        </is>
+      </c>
+      <c r="B21" s="36" t="inlineStr">
+        <is>
+          <t>m of coastline</t>
+        </is>
+      </c>
+      <c r="C21" s="38" t="n"/>
+      <c r="D21" s="38" t="n"/>
+      <c r="E21" s="38" t="n"/>
+      <c r="F21" s="38" t="n"/>
+      <c r="G21" s="38" t="n"/>
+      <c r="H21" s="38" t="n"/>
+      <c r="I21" s="37" t="n"/>
+      <c r="J21" s="37" t="n"/>
+      <c r="K21" s="37" t="n"/>
+      <c r="L21" s="38" t="n"/>
+      <c r="M21" s="38" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="35" t="inlineStr">
+        <is>
+          <t>Nursery habitat support</t>
+        </is>
+      </c>
+      <c r="B22" s="36" t="inlineStr">
+        <is>
+          <t>kg fish/yr</t>
+        </is>
+      </c>
+      <c r="C22" s="38" t="n"/>
+      <c r="D22" s="38" t="n"/>
+      <c r="E22" s="38" t="n"/>
+      <c r="F22" s="38" t="n"/>
+      <c r="G22" s="38" t="n"/>
+      <c r="H22" s="38" t="n"/>
+      <c r="I22" s="37" t="n"/>
+      <c r="J22" s="37" t="n"/>
+      <c r="K22" s="37" t="n"/>
+      <c r="L22" s="38" t="n"/>
+      <c r="M22" s="38" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="44" t="inlineStr">
+        <is>
+          <t>Cultural services (SEEA EA 6.6)</t>
+        </is>
+      </c>
+      <c r="B23" s="45" t="n"/>
+      <c r="C23" s="45" t="n"/>
+      <c r="D23" s="45" t="n"/>
+      <c r="E23" s="45" t="n"/>
+      <c r="F23" s="45" t="n"/>
+      <c r="G23" s="45" t="n"/>
+      <c r="H23" s="45" t="n"/>
+      <c r="I23" s="45" t="n"/>
+      <c r="J23" s="45" t="n"/>
+      <c r="K23" s="45" t="n"/>
+      <c r="L23" s="45" t="n"/>
+      <c r="M23" s="45" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="35" t="inlineStr">
+        <is>
+          <t>Recreation &amp; tourism</t>
+        </is>
+      </c>
+      <c r="B24" s="36" t="inlineStr">
         <is>
           <t>visitors/yr</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Gleaning</t>
-        </is>
-      </c>
-      <c r="B9" s="27" t="inlineStr">
+      <c r="C24" s="38" t="n"/>
+      <c r="D24" s="38" t="n"/>
+      <c r="E24" s="38" t="n"/>
+      <c r="F24" s="38" t="n"/>
+      <c r="G24" s="38" t="n"/>
+      <c r="H24" s="38" t="n"/>
+      <c r="I24" s="37" t="n"/>
+      <c r="J24" s="37" t="n"/>
+      <c r="K24" s="37" t="n"/>
+      <c r="L24" s="38" t="n"/>
+      <c r="M24" s="38" t="n"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="35" t="inlineStr">
+        <is>
+          <t>Gleaning (subsistence harvest)</t>
+        </is>
+      </c>
+      <c r="B25" s="36" t="inlineStr">
         <is>
           <t>hours/yr</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="28" t="inlineStr">
-        <is>
-          <t>Note: Total supply must equal Total use for each service (accounting identity)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>Combined Monetary Supply and Use Table (USD/yr)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="n"/>
-      <c r="B15" s="21" t="n"/>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>SUPPLY (by ecosystem)</t>
-        </is>
-      </c>
-      <c r="D15" s="22" t="n"/>
-      <c r="E15" s="22" t="n"/>
-      <c r="F15" s="22" t="n"/>
-      <c r="G15" s="23" t="inlineStr">
-        <is>
-          <t>USE (by beneficiary)</t>
-        </is>
-      </c>
-      <c r="H15" s="21" t="n"/>
-      <c r="I15" s="21" t="n"/>
-      <c r="J15" s="21" t="n"/>
-      <c r="K15" s="21" t="n"/>
-      <c r="L15" s="21" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="24" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="C16" s="25" t="inlineStr">
-        <is>
-          <t>Coral reefs</t>
-        </is>
-      </c>
-      <c r="D16" s="25" t="inlineStr">
-        <is>
-          <t>Seagrass</t>
-        </is>
-      </c>
-      <c r="E16" s="25" t="inlineStr">
-        <is>
-          <t>Mangroves</t>
-        </is>
-      </c>
-      <c r="F16" s="25" t="inlineStr">
-        <is>
-          <t>Total supply</t>
-        </is>
-      </c>
-      <c r="G16" s="26" t="inlineStr">
-        <is>
-          <t>Fisheries</t>
-        </is>
-      </c>
-      <c r="H16" s="26" t="inlineStr">
-        <is>
-          <t>Tourism</t>
-        </is>
-      </c>
-      <c r="I16" s="26" t="inlineStr">
-        <is>
-          <t>Coastal HH</t>
-        </is>
-      </c>
-      <c r="J16" s="26" t="inlineStr">
-        <is>
-          <t>Govt</t>
-        </is>
-      </c>
-      <c r="K16" s="26" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="L16" s="26" t="inlineStr">
-        <is>
-          <t>Total use</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Fish provisioning</t>
-        </is>
-      </c>
-      <c r="B17" s="27" t="inlineStr">
-        <is>
-          <t>USD/yr</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="7" t="n"/>
-      <c r="I17" s="7" t="n"/>
-      <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Carbon sequestration</t>
-        </is>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
-        <is>
-          <t>USD/yr</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
-      <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="n"/>
-      <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Coastal protection</t>
-        </is>
-      </c>
-      <c r="B19" s="27" t="inlineStr">
-        <is>
-          <t>USD/yr</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
-      <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="7" t="n"/>
-      <c r="I19" s="7" t="n"/>
-      <c r="J19" s="7" t="n"/>
-      <c r="K19" s="7" t="n"/>
-      <c r="L19" s="7" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Nursery habitat</t>
-        </is>
-      </c>
-      <c r="B20" s="27" t="inlineStr">
-        <is>
-          <t>USD/yr</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
-      <c r="I20" s="7" t="n"/>
-      <c r="J20" s="7" t="n"/>
-      <c r="K20" s="7" t="n"/>
-      <c r="L20" s="7" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Recreation</t>
-        </is>
-      </c>
-      <c r="B21" s="27" t="inlineStr">
-        <is>
-          <t>USD/yr</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="7" t="n"/>
-      <c r="I21" s="7" t="n"/>
-      <c r="J21" s="7" t="n"/>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Gleaning</t>
-        </is>
-      </c>
-      <c r="B22" s="27" t="inlineStr">
-        <is>
-          <t>USD/yr</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
-      <c r="I22" s="7" t="n"/>
-      <c r="J22" s="7" t="n"/>
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
+      <c r="C25" s="38" t="n"/>
+      <c r="D25" s="38" t="n"/>
+      <c r="E25" s="38" t="n"/>
+      <c r="F25" s="38" t="n"/>
+      <c r="G25" s="38" t="n"/>
+      <c r="H25" s="38" t="n"/>
+      <c r="I25" s="37" t="n"/>
+      <c r="J25" s="37" t="n"/>
+      <c r="K25" s="37" t="n"/>
+      <c r="L25" s="38" t="n"/>
+      <c r="M25" s="38" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="46" t="inlineStr">
+        <is>
+          <t>Note: Format follows SEEA EA Table 7.1 (supply and use of ecosystem services). Carbon sequestration use allocated to Global/Exports as the benefit accrues globally.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="G15:L15"/>
-    <mergeCell ref="G2:L2"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A14:L14"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="A12:L12"/>
+  <mergeCells count="15">
+    <mergeCell ref="A28:M28"/>
+    <mergeCell ref="A19:M19"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="C2:H2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A23:M23"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="A17:M17"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="A10:M10"/>
+    <mergeCell ref="C15:H15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rebuild SUT as proper single SEEA EA Table 7.1 format
One integrated table with SUPPLY on top and USE on bottom,
sharing the same columns (economic units + ecosystem types):

SUPPLY half: ecosystem type columns FILLED (mint background),
  economic unit columns EMPTY (grey) -- ecosystems supply services
USE half: economic unit columns FILLED (light blue background),
  ecosystem type columns EMPTY (grey) -- economic units use services

This matches SEEA EA Table 7.1a/7.1b exactly:
- Supply shows where services come from (ecosystem assets)
- Use shows who benefits (industries, households, government, exports)
- Same services listed in both halves
- Total supply = Total use (accounting identity)

Updated in example Excel (filled), template Excel (blank with yellow
input cells and grey blocked cells), exercise Excel, and print
notebook copies.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/s-s-event-bogor/print-notebooks/03-services/10-template.xlsx
+++ b/s-s-event-bogor/print-notebooks/03-services/10-template.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monetary Use" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculations" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combined Supply-Use" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUT (Supply-Use Table)" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,8 +131,39 @@
       <color rgb="00404040"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0030302F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="0030302F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="0030302F"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -173,6 +204,36 @@
       <patternFill patternType="solid">
         <fgColor rgb="00B2D8D8"/>
         <bgColor rgb="00B2D8D8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00404040"/>
+        <bgColor rgb="00404040"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A8D5C2"/>
+        <bgColor rgb="00A8D5C2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007FBCBD"/>
+        <bgColor rgb="007FBCBD"/>
       </patternFill>
     </fill>
   </fills>
@@ -246,7 +307,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -351,6 +412,42 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2377,10 +2474,11 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="003B9C7B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2389,653 +2487,592 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="29" t="inlineStr">
-        <is>
-          <t>SUPPLY TABLE (Table 7.1a)</t>
-        </is>
-      </c>
-      <c r="B1" s="30" t="n"/>
-      <c r="C1" s="30" t="n"/>
-      <c r="D1" s="30" t="n"/>
-      <c r="E1" s="30" t="n"/>
-      <c r="F1" s="30" t="n"/>
-      <c r="G1" s="30" t="n"/>
-      <c r="H1" s="30" t="n"/>
-      <c r="I1" s="30" t="n"/>
-      <c r="J1" s="30" t="n"/>
-      <c r="K1" s="30" t="n"/>
-      <c r="L1" s="30" t="n"/>
-      <c r="M1" s="30" t="n"/>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="22" t="n"/>
-      <c r="B2" s="22" t="n"/>
-      <c r="C2" s="31" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="47" t="inlineStr">
+        <is>
+          <t>Ecosystem Services Supply-Use Table (SEEA EA Table 7.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="48" t="inlineStr">
+        <is>
+          <t>Integrated supply and use account for ocean ecosystem services</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="49" t="inlineStr"/>
+      <c r="B4" s="49" t="inlineStr"/>
+      <c r="C4" s="49" t="inlineStr">
         <is>
           <t>Economic units</t>
         </is>
       </c>
-      <c r="D2" s="22" t="n"/>
-      <c r="E2" s="22" t="n"/>
-      <c r="F2" s="22" t="n"/>
-      <c r="G2" s="22" t="n"/>
-      <c r="H2" s="22" t="n"/>
-      <c r="I2" s="31" t="inlineStr">
+      <c r="D4" s="50" t="n"/>
+      <c r="E4" s="50" t="n"/>
+      <c r="F4" s="50" t="n"/>
+      <c r="G4" s="50" t="n"/>
+      <c r="H4" s="51" t="n"/>
+      <c r="I4" s="49" t="inlineStr">
         <is>
           <t>Ecosystem types</t>
         </is>
       </c>
-      <c r="J2" s="22" t="n"/>
-      <c r="K2" s="22" t="n"/>
-      <c r="L2" s="22" t="n"/>
-      <c r="M2" s="22" t="n"/>
-    </row>
-    <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="32" t="inlineStr">
+      <c r="J4" s="50" t="n"/>
+      <c r="K4" s="51" t="n"/>
+      <c r="L4" s="49" t="inlineStr"/>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="49" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="B3" s="32" t="inlineStr">
+      <c r="B5" s="49" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="C3" s="32" t="inlineStr">
-        <is>
-          <t>Fisheries</t>
-        </is>
-      </c>
-      <c r="D3" s="32" t="inlineStr">
-        <is>
-          <t>Tourism</t>
-        </is>
-      </c>
-      <c r="E3" s="32" t="inlineStr">
-        <is>
-          <t>Other industry</t>
-        </is>
-      </c>
-      <c r="F3" s="32" t="inlineStr">
+      <c r="C5" s="49" t="inlineStr">
+        <is>
+          <t>Fisheries
+sector</t>
+        </is>
+      </c>
+      <c r="D5" s="49" t="inlineStr">
+        <is>
+          <t>Tourism
+sector</t>
+        </is>
+      </c>
+      <c r="E5" s="49" t="inlineStr">
+        <is>
+          <t>Other
+industries</t>
+        </is>
+      </c>
+      <c r="F5" s="49" t="inlineStr">
         <is>
           <t>Households</t>
         </is>
       </c>
-      <c r="G3" s="32" t="inlineStr">
-        <is>
-          <t>Govt</t>
-        </is>
-      </c>
-      <c r="H3" s="32" t="inlineStr">
-        <is>
-          <t>Global/Exports</t>
-        </is>
-      </c>
-      <c r="I3" s="32" t="inlineStr">
+      <c r="G5" s="49" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="H5" s="49" t="inlineStr">
+        <is>
+          <t>Exports /
+Global</t>
+        </is>
+      </c>
+      <c r="I5" s="49" t="inlineStr">
         <is>
           <t>Coral reefs
 (M1.3)</t>
         </is>
       </c>
-      <c r="J3" s="32" t="inlineStr">
-        <is>
-          <t>Seagrass meadows
+      <c r="J5" s="49" t="inlineStr">
+        <is>
+          <t>Seagrass
+meadows
 (M1.1)</t>
         </is>
       </c>
-      <c r="K3" s="32" t="inlineStr">
+      <c r="K5" s="49" t="inlineStr">
         <is>
           <t>Mangroves
 (MFT1.2)</t>
         </is>
       </c>
-      <c r="L3" s="32" t="inlineStr">
-        <is>
-          <t>Total ecosystem</t>
-        </is>
-      </c>
-      <c r="M3" s="32" t="inlineStr">
+      <c r="L5" s="49" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="33" t="inlineStr">
-        <is>
-          <t>Provisioning services (SEEA EA 6.1)</t>
-        </is>
-      </c>
-      <c r="B4" s="34" t="n"/>
-      <c r="C4" s="34" t="n"/>
-      <c r="D4" s="34" t="n"/>
-      <c r="E4" s="34" t="n"/>
-      <c r="F4" s="34" t="n"/>
-      <c r="G4" s="34" t="n"/>
-      <c r="H4" s="34" t="n"/>
-      <c r="I4" s="34" t="n"/>
-      <c r="J4" s="34" t="n"/>
-      <c r="K4" s="34" t="n"/>
-      <c r="L4" s="34" t="n"/>
-      <c r="M4" s="34" t="n"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="35" t="inlineStr">
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="52" t="inlineStr">
+        <is>
+          <t>SUPPLY</t>
+        </is>
+      </c>
+      <c r="B6" s="50" t="n"/>
+      <c r="C6" s="50" t="n"/>
+      <c r="D6" s="50" t="n"/>
+      <c r="E6" s="50" t="n"/>
+      <c r="F6" s="50" t="n"/>
+      <c r="G6" s="50" t="n"/>
+      <c r="H6" s="50" t="n"/>
+      <c r="I6" s="50" t="n"/>
+      <c r="J6" s="50" t="n"/>
+      <c r="K6" s="50" t="n"/>
+      <c r="L6" s="51" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="53" t="inlineStr">
+        <is>
+          <t>Provisioning (SEEA EA 6.1)</t>
+        </is>
+      </c>
+      <c r="B7" s="50" t="n"/>
+      <c r="C7" s="50" t="n"/>
+      <c r="D7" s="50" t="n"/>
+      <c r="E7" s="50" t="n"/>
+      <c r="F7" s="50" t="n"/>
+      <c r="G7" s="50" t="n"/>
+      <c r="H7" s="50" t="n"/>
+      <c r="I7" s="50" t="n"/>
+      <c r="J7" s="50" t="n"/>
+      <c r="K7" s="50" t="n"/>
+      <c r="L7" s="51" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="54" t="inlineStr">
         <is>
           <t>Fish provisioning</t>
         </is>
       </c>
-      <c r="B5" s="36" t="inlineStr">
-        <is>
-          <t>kg/yr</t>
-        </is>
-      </c>
-      <c r="C5" s="37" t="n"/>
-      <c r="D5" s="37" t="n"/>
-      <c r="E5" s="37" t="n"/>
-      <c r="F5" s="37" t="n"/>
-      <c r="G5" s="37" t="n"/>
-      <c r="H5" s="37" t="n"/>
-      <c r="I5" s="38" t="n"/>
-      <c r="J5" s="38" t="n"/>
-      <c r="K5" s="38" t="n"/>
-      <c r="L5" s="38" t="n"/>
-      <c r="M5" s="38" t="n"/>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="33" t="inlineStr">
-        <is>
-          <t>Regulating &amp; maintenance services (SEEA EA 6.2-6.5)</t>
-        </is>
-      </c>
-      <c r="B6" s="34" t="n"/>
-      <c r="C6" s="34" t="n"/>
-      <c r="D6" s="34" t="n"/>
-      <c r="E6" s="34" t="n"/>
-      <c r="F6" s="34" t="n"/>
-      <c r="G6" s="34" t="n"/>
-      <c r="H6" s="34" t="n"/>
-      <c r="I6" s="34" t="n"/>
-      <c r="J6" s="34" t="n"/>
-      <c r="K6" s="34" t="n"/>
-      <c r="L6" s="34" t="n"/>
-      <c r="M6" s="34" t="n"/>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="35" t="inlineStr">
+      <c r="B8" s="55" t="inlineStr">
+        <is>
+          <t>tonnes</t>
+        </is>
+      </c>
+      <c r="C8" s="56" t="n"/>
+      <c r="D8" s="56" t="n"/>
+      <c r="E8" s="56" t="n"/>
+      <c r="F8" s="56" t="n"/>
+      <c r="G8" s="56" t="n"/>
+      <c r="H8" s="56" t="n"/>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="57">
+        <f>SUM(I8:K8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="53" t="inlineStr">
+        <is>
+          <t>Regulating (SEEA EA 6.2-6.5)</t>
+        </is>
+      </c>
+      <c r="B9" s="50" t="n"/>
+      <c r="C9" s="50" t="n"/>
+      <c r="D9" s="50" t="n"/>
+      <c r="E9" s="50" t="n"/>
+      <c r="F9" s="50" t="n"/>
+      <c r="G9" s="50" t="n"/>
+      <c r="H9" s="50" t="n"/>
+      <c r="I9" s="50" t="n"/>
+      <c r="J9" s="50" t="n"/>
+      <c r="K9" s="50" t="n"/>
+      <c r="L9" s="51" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="54" t="inlineStr">
         <is>
           <t>Carbon sequestration</t>
         </is>
       </c>
-      <c r="B7" s="36" t="inlineStr">
-        <is>
-          <t>Mg CO₂/yr</t>
-        </is>
-      </c>
-      <c r="C7" s="37" t="n"/>
-      <c r="D7" s="37" t="n"/>
-      <c r="E7" s="37" t="n"/>
-      <c r="F7" s="37" t="n"/>
-      <c r="G7" s="37" t="n"/>
-      <c r="H7" s="37" t="n"/>
-      <c r="I7" s="38" t="n"/>
-      <c r="J7" s="38" t="n"/>
-      <c r="K7" s="38" t="n"/>
-      <c r="L7" s="38" t="n"/>
-      <c r="M7" s="38" t="n"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="35" t="inlineStr">
+      <c r="B10" s="55" t="inlineStr">
+        <is>
+          <t>tCO₂/yr</t>
+        </is>
+      </c>
+      <c r="C10" s="56" t="n"/>
+      <c r="D10" s="56" t="n"/>
+      <c r="E10" s="56" t="n"/>
+      <c r="F10" s="56" t="n"/>
+      <c r="G10" s="56" t="n"/>
+      <c r="H10" s="56" t="n"/>
+      <c r="I10" s="7" t="n"/>
+      <c r="J10" s="7" t="n"/>
+      <c r="K10" s="7" t="n"/>
+      <c r="L10" s="57">
+        <f>SUM(I10:K10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="54" t="inlineStr">
         <is>
           <t>Coastal protection</t>
         </is>
       </c>
-      <c r="B8" s="36" t="inlineStr">
-        <is>
-          <t>m of coastline</t>
-        </is>
-      </c>
-      <c r="C8" s="37" t="n"/>
-      <c r="D8" s="37" t="n"/>
-      <c r="E8" s="37" t="n"/>
-      <c r="F8" s="37" t="n"/>
-      <c r="G8" s="37" t="n"/>
-      <c r="H8" s="37" t="n"/>
-      <c r="I8" s="38" t="n"/>
-      <c r="J8" s="38" t="n"/>
-      <c r="K8" s="38" t="n"/>
-      <c r="L8" s="38" t="n"/>
-      <c r="M8" s="38" t="n"/>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="35" t="inlineStr">
-        <is>
-          <t>Nursery habitat support</t>
-        </is>
-      </c>
-      <c r="B9" s="36" t="inlineStr">
-        <is>
-          <t>kg fish/yr</t>
-        </is>
-      </c>
-      <c r="C9" s="37" t="n"/>
-      <c r="D9" s="37" t="n"/>
-      <c r="E9" s="37" t="n"/>
-      <c r="F9" s="37" t="n"/>
-      <c r="G9" s="37" t="n"/>
-      <c r="H9" s="37" t="n"/>
-      <c r="I9" s="38" t="n"/>
-      <c r="J9" s="38" t="n"/>
-      <c r="K9" s="38" t="n"/>
-      <c r="L9" s="38" t="n"/>
-      <c r="M9" s="38" t="n"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="33" t="inlineStr">
-        <is>
-          <t>Cultural services (SEEA EA 6.6)</t>
-        </is>
-      </c>
-      <c r="B10" s="34" t="n"/>
-      <c r="C10" s="34" t="n"/>
-      <c r="D10" s="34" t="n"/>
-      <c r="E10" s="34" t="n"/>
-      <c r="F10" s="34" t="n"/>
-      <c r="G10" s="34" t="n"/>
-      <c r="H10" s="34" t="n"/>
-      <c r="I10" s="34" t="n"/>
-      <c r="J10" s="34" t="n"/>
-      <c r="K10" s="34" t="n"/>
-      <c r="L10" s="34" t="n"/>
-      <c r="M10" s="34" t="n"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="35" t="inlineStr">
-        <is>
-          <t>Recreation &amp; tourism</t>
-        </is>
-      </c>
-      <c r="B11" s="36" t="inlineStr">
-        <is>
-          <t>visitors/yr</t>
-        </is>
-      </c>
-      <c r="C11" s="37" t="n"/>
-      <c r="D11" s="37" t="n"/>
-      <c r="E11" s="37" t="n"/>
-      <c r="F11" s="37" t="n"/>
-      <c r="G11" s="37" t="n"/>
-      <c r="H11" s="37" t="n"/>
-      <c r="I11" s="38" t="n"/>
-      <c r="J11" s="38" t="n"/>
-      <c r="K11" s="38" t="n"/>
-      <c r="L11" s="38" t="n"/>
-      <c r="M11" s="38" t="n"/>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="35" t="inlineStr">
-        <is>
-          <t>Gleaning (subsistence harvest)</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="inlineStr">
-        <is>
-          <t>hours/yr</t>
-        </is>
-      </c>
-      <c r="C12" s="37" t="n"/>
-      <c r="D12" s="37" t="n"/>
-      <c r="E12" s="37" t="n"/>
-      <c r="F12" s="37" t="n"/>
-      <c r="G12" s="37" t="n"/>
-      <c r="H12" s="37" t="n"/>
-      <c r="I12" s="38" t="n"/>
-      <c r="J12" s="38" t="n"/>
-      <c r="K12" s="38" t="n"/>
-      <c r="L12" s="38" t="n"/>
-      <c r="M12" s="38" t="n"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="39" t="inlineStr">
-        <is>
-          <t>USE TABLE (Table 7.1b)</t>
-        </is>
-      </c>
-      <c r="B14" s="40" t="n"/>
-      <c r="C14" s="40" t="n"/>
-      <c r="D14" s="40" t="n"/>
-      <c r="E14" s="40" t="n"/>
-      <c r="F14" s="40" t="n"/>
-      <c r="G14" s="40" t="n"/>
-      <c r="H14" s="40" t="n"/>
-      <c r="I14" s="40" t="n"/>
-      <c r="J14" s="40" t="n"/>
-      <c r="K14" s="40" t="n"/>
-      <c r="L14" s="40" t="n"/>
-      <c r="M14" s="40" t="n"/>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="41" t="n"/>
-      <c r="B15" s="41" t="n"/>
-      <c r="C15" s="42" t="inlineStr">
-        <is>
-          <t>Economic units</t>
-        </is>
-      </c>
-      <c r="D15" s="41" t="n"/>
-      <c r="E15" s="41" t="n"/>
-      <c r="F15" s="41" t="n"/>
-      <c r="G15" s="41" t="n"/>
-      <c r="H15" s="41" t="n"/>
-      <c r="I15" s="42" t="inlineStr">
-        <is>
-          <t>Ecosystem types</t>
-        </is>
-      </c>
-      <c r="J15" s="41" t="n"/>
-      <c r="K15" s="41" t="n"/>
-      <c r="L15" s="41" t="n"/>
-      <c r="M15" s="41" t="n"/>
-    </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="43" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="B16" s="43" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="C16" s="43" t="inlineStr">
-        <is>
-          <t>Fisheries</t>
-        </is>
-      </c>
-      <c r="D16" s="43" t="inlineStr">
-        <is>
-          <t>Tourism</t>
-        </is>
-      </c>
-      <c r="E16" s="43" t="inlineStr">
-        <is>
-          <t>Other industry</t>
-        </is>
-      </c>
-      <c r="F16" s="43" t="inlineStr">
-        <is>
-          <t>Households</t>
-        </is>
-      </c>
-      <c r="G16" s="43" t="inlineStr">
-        <is>
-          <t>Govt</t>
-        </is>
-      </c>
-      <c r="H16" s="43" t="inlineStr">
-        <is>
-          <t>Global/Exports</t>
-        </is>
-      </c>
-      <c r="I16" s="43" t="inlineStr">
-        <is>
-          <t>Coral reefs
-(M1.3)</t>
-        </is>
-      </c>
-      <c r="J16" s="43" t="inlineStr">
-        <is>
-          <t>Seagrass meadows
-(M1.1)</t>
-        </is>
-      </c>
-      <c r="K16" s="43" t="inlineStr">
-        <is>
-          <t>Mangroves
-(MFT1.2)</t>
-        </is>
-      </c>
-      <c r="L16" s="43" t="inlineStr">
-        <is>
-          <t>Total ecosystem</t>
-        </is>
-      </c>
-      <c r="M16" s="43" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="44" t="inlineStr">
-        <is>
-          <t>Provisioning services (SEEA EA 6.1)</t>
-        </is>
-      </c>
-      <c r="B17" s="45" t="n"/>
-      <c r="C17" s="45" t="n"/>
-      <c r="D17" s="45" t="n"/>
-      <c r="E17" s="45" t="n"/>
-      <c r="F17" s="45" t="n"/>
-      <c r="G17" s="45" t="n"/>
-      <c r="H17" s="45" t="n"/>
-      <c r="I17" s="45" t="n"/>
-      <c r="J17" s="45" t="n"/>
-      <c r="K17" s="45" t="n"/>
-      <c r="L17" s="45" t="n"/>
-      <c r="M17" s="45" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="35" t="inlineStr">
+      <c r="B11" s="55" t="inlineStr">
+        <is>
+          <t>USD thousands</t>
+        </is>
+      </c>
+      <c r="C11" s="56" t="n"/>
+      <c r="D11" s="56" t="n"/>
+      <c r="E11" s="56" t="n"/>
+      <c r="F11" s="56" t="n"/>
+      <c r="G11" s="56" t="n"/>
+      <c r="H11" s="56" t="n"/>
+      <c r="I11" s="7" t="n"/>
+      <c r="J11" s="7" t="n"/>
+      <c r="K11" s="7" t="n"/>
+      <c r="L11" s="57">
+        <f>SUM(I11:K11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="54" t="inlineStr">
+        <is>
+          <t>Nursery habitat</t>
+        </is>
+      </c>
+      <c r="B12" s="55" t="inlineStr">
+        <is>
+          <t>hectares</t>
+        </is>
+      </c>
+      <c r="C12" s="56" t="n"/>
+      <c r="D12" s="56" t="n"/>
+      <c r="E12" s="56" t="n"/>
+      <c r="F12" s="56" t="n"/>
+      <c r="G12" s="56" t="n"/>
+      <c r="H12" s="56" t="n"/>
+      <c r="I12" s="7" t="n"/>
+      <c r="J12" s="7" t="n"/>
+      <c r="K12" s="7" t="n"/>
+      <c r="L12" s="57">
+        <f>SUM(I12:K12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="53" t="inlineStr">
+        <is>
+          <t>Cultural (SEEA EA 6.6)</t>
+        </is>
+      </c>
+      <c r="B13" s="50" t="n"/>
+      <c r="C13" s="50" t="n"/>
+      <c r="D13" s="50" t="n"/>
+      <c r="E13" s="50" t="n"/>
+      <c r="F13" s="50" t="n"/>
+      <c r="G13" s="50" t="n"/>
+      <c r="H13" s="50" t="n"/>
+      <c r="I13" s="50" t="n"/>
+      <c r="J13" s="50" t="n"/>
+      <c r="K13" s="50" t="n"/>
+      <c r="L13" s="51" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="54" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="B14" s="55" t="inlineStr">
+        <is>
+          <t>visitor-days</t>
+        </is>
+      </c>
+      <c r="C14" s="56" t="n"/>
+      <c r="D14" s="56" t="n"/>
+      <c r="E14" s="56" t="n"/>
+      <c r="F14" s="56" t="n"/>
+      <c r="G14" s="56" t="n"/>
+      <c r="H14" s="56" t="n"/>
+      <c r="I14" s="7" t="n"/>
+      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="7" t="n"/>
+      <c r="L14" s="57">
+        <f>SUM(I14:K14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="54" t="inlineStr">
+        <is>
+          <t>Gleaning</t>
+        </is>
+      </c>
+      <c r="B15" s="55" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="C15" s="56" t="n"/>
+      <c r="D15" s="56" t="n"/>
+      <c r="E15" s="56" t="n"/>
+      <c r="F15" s="56" t="n"/>
+      <c r="G15" s="56" t="n"/>
+      <c r="H15" s="56" t="n"/>
+      <c r="I15" s="7" t="n"/>
+      <c r="J15" s="7" t="n"/>
+      <c r="K15" s="7" t="n"/>
+      <c r="L15" s="57">
+        <f>SUM(I15:K15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="58" t="n"/>
+      <c r="B16" s="58" t="n"/>
+      <c r="C16" s="58" t="n"/>
+      <c r="D16" s="58" t="n"/>
+      <c r="E16" s="58" t="n"/>
+      <c r="F16" s="58" t="n"/>
+      <c r="G16" s="58" t="n"/>
+      <c r="H16" s="58" t="n"/>
+      <c r="I16" s="58" t="n"/>
+      <c r="J16" s="58" t="n"/>
+      <c r="K16" s="58" t="n"/>
+      <c r="L16" s="58" t="n"/>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="59" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="B17" s="50" t="n"/>
+      <c r="C17" s="50" t="n"/>
+      <c r="D17" s="50" t="n"/>
+      <c r="E17" s="50" t="n"/>
+      <c r="F17" s="50" t="n"/>
+      <c r="G17" s="50" t="n"/>
+      <c r="H17" s="50" t="n"/>
+      <c r="I17" s="50" t="n"/>
+      <c r="J17" s="50" t="n"/>
+      <c r="K17" s="50" t="n"/>
+      <c r="L17" s="51" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="60" t="inlineStr">
+        <is>
+          <t>Provisioning (SEEA EA 6.1)</t>
+        </is>
+      </c>
+      <c r="B18" s="50" t="n"/>
+      <c r="C18" s="50" t="n"/>
+      <c r="D18" s="50" t="n"/>
+      <c r="E18" s="50" t="n"/>
+      <c r="F18" s="50" t="n"/>
+      <c r="G18" s="50" t="n"/>
+      <c r="H18" s="50" t="n"/>
+      <c r="I18" s="50" t="n"/>
+      <c r="J18" s="50" t="n"/>
+      <c r="K18" s="50" t="n"/>
+      <c r="L18" s="51" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="54" t="inlineStr">
         <is>
           <t>Fish provisioning</t>
         </is>
       </c>
-      <c r="B18" s="36" t="inlineStr">
-        <is>
-          <t>kg/yr</t>
-        </is>
-      </c>
-      <c r="C18" s="38" t="n"/>
-      <c r="D18" s="38" t="n"/>
-      <c r="E18" s="38" t="n"/>
-      <c r="F18" s="38" t="n"/>
-      <c r="G18" s="38" t="n"/>
-      <c r="H18" s="38" t="n"/>
-      <c r="I18" s="37" t="n"/>
-      <c r="J18" s="37" t="n"/>
-      <c r="K18" s="37" t="n"/>
-      <c r="L18" s="38" t="n"/>
-      <c r="M18" s="38" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="44" t="inlineStr">
-        <is>
-          <t>Regulating &amp; maintenance services (SEEA EA 6.2-6.5)</t>
-        </is>
-      </c>
-      <c r="B19" s="45" t="n"/>
-      <c r="C19" s="45" t="n"/>
-      <c r="D19" s="45" t="n"/>
-      <c r="E19" s="45" t="n"/>
-      <c r="F19" s="45" t="n"/>
-      <c r="G19" s="45" t="n"/>
-      <c r="H19" s="45" t="n"/>
-      <c r="I19" s="45" t="n"/>
-      <c r="J19" s="45" t="n"/>
-      <c r="K19" s="45" t="n"/>
-      <c r="L19" s="45" t="n"/>
-      <c r="M19" s="45" t="n"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="35" t="inlineStr">
+      <c r="B19" s="55" t="inlineStr">
+        <is>
+          <t>tonnes</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="56" t="n"/>
+      <c r="J19" s="56" t="n"/>
+      <c r="K19" s="56" t="n"/>
+      <c r="L19" s="57">
+        <f>SUM(C19:H19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="60" t="inlineStr">
+        <is>
+          <t>Regulating (SEEA EA 6.2-6.5)</t>
+        </is>
+      </c>
+      <c r="B20" s="50" t="n"/>
+      <c r="C20" s="50" t="n"/>
+      <c r="D20" s="50" t="n"/>
+      <c r="E20" s="50" t="n"/>
+      <c r="F20" s="50" t="n"/>
+      <c r="G20" s="50" t="n"/>
+      <c r="H20" s="50" t="n"/>
+      <c r="I20" s="50" t="n"/>
+      <c r="J20" s="50" t="n"/>
+      <c r="K20" s="50" t="n"/>
+      <c r="L20" s="51" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="54" t="inlineStr">
         <is>
           <t>Carbon sequestration</t>
         </is>
       </c>
-      <c r="B20" s="36" t="inlineStr">
-        <is>
-          <t>Mg CO₂/yr</t>
-        </is>
-      </c>
-      <c r="C20" s="38" t="n"/>
-      <c r="D20" s="38" t="n"/>
-      <c r="E20" s="38" t="n"/>
-      <c r="F20" s="38" t="n"/>
-      <c r="G20" s="38" t="n"/>
-      <c r="H20" s="38" t="n"/>
-      <c r="I20" s="37" t="n"/>
-      <c r="J20" s="37" t="n"/>
-      <c r="K20" s="37" t="n"/>
-      <c r="L20" s="38" t="n"/>
-      <c r="M20" s="38" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="35" t="inlineStr">
+      <c r="B21" s="55" t="inlineStr">
+        <is>
+          <t>tCO₂/yr</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="56" t="n"/>
+      <c r="J21" s="56" t="n"/>
+      <c r="K21" s="56" t="n"/>
+      <c r="L21" s="57">
+        <f>SUM(C21:H21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="54" t="inlineStr">
         <is>
           <t>Coastal protection</t>
         </is>
       </c>
-      <c r="B21" s="36" t="inlineStr">
-        <is>
-          <t>m of coastline</t>
-        </is>
-      </c>
-      <c r="C21" s="38" t="n"/>
-      <c r="D21" s="38" t="n"/>
-      <c r="E21" s="38" t="n"/>
-      <c r="F21" s="38" t="n"/>
-      <c r="G21" s="38" t="n"/>
-      <c r="H21" s="38" t="n"/>
-      <c r="I21" s="37" t="n"/>
-      <c r="J21" s="37" t="n"/>
-      <c r="K21" s="37" t="n"/>
-      <c r="L21" s="38" t="n"/>
-      <c r="M21" s="38" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="35" t="inlineStr">
-        <is>
-          <t>Nursery habitat support</t>
-        </is>
-      </c>
-      <c r="B22" s="36" t="inlineStr">
-        <is>
-          <t>kg fish/yr</t>
-        </is>
-      </c>
-      <c r="C22" s="38" t="n"/>
-      <c r="D22" s="38" t="n"/>
-      <c r="E22" s="38" t="n"/>
-      <c r="F22" s="38" t="n"/>
-      <c r="G22" s="38" t="n"/>
-      <c r="H22" s="38" t="n"/>
-      <c r="I22" s="37" t="n"/>
-      <c r="J22" s="37" t="n"/>
-      <c r="K22" s="37" t="n"/>
-      <c r="L22" s="38" t="n"/>
-      <c r="M22" s="38" t="n"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="44" t="inlineStr">
-        <is>
-          <t>Cultural services (SEEA EA 6.6)</t>
-        </is>
-      </c>
-      <c r="B23" s="45" t="n"/>
-      <c r="C23" s="45" t="n"/>
-      <c r="D23" s="45" t="n"/>
-      <c r="E23" s="45" t="n"/>
-      <c r="F23" s="45" t="n"/>
-      <c r="G23" s="45" t="n"/>
-      <c r="H23" s="45" t="n"/>
-      <c r="I23" s="45" t="n"/>
-      <c r="J23" s="45" t="n"/>
-      <c r="K23" s="45" t="n"/>
-      <c r="L23" s="45" t="n"/>
-      <c r="M23" s="45" t="n"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="35" t="inlineStr">
-        <is>
-          <t>Recreation &amp; tourism</t>
-        </is>
-      </c>
-      <c r="B24" s="36" t="inlineStr">
-        <is>
-          <t>visitors/yr</t>
-        </is>
-      </c>
-      <c r="C24" s="38" t="n"/>
-      <c r="D24" s="38" t="n"/>
-      <c r="E24" s="38" t="n"/>
-      <c r="F24" s="38" t="n"/>
-      <c r="G24" s="38" t="n"/>
-      <c r="H24" s="38" t="n"/>
-      <c r="I24" s="37" t="n"/>
-      <c r="J24" s="37" t="n"/>
-      <c r="K24" s="37" t="n"/>
-      <c r="L24" s="38" t="n"/>
-      <c r="M24" s="38" t="n"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="35" t="inlineStr">
-        <is>
-          <t>Gleaning (subsistence harvest)</t>
-        </is>
-      </c>
-      <c r="B25" s="36" t="inlineStr">
-        <is>
-          <t>hours/yr</t>
-        </is>
-      </c>
-      <c r="C25" s="38" t="n"/>
-      <c r="D25" s="38" t="n"/>
-      <c r="E25" s="38" t="n"/>
-      <c r="F25" s="38" t="n"/>
-      <c r="G25" s="38" t="n"/>
-      <c r="H25" s="38" t="n"/>
-      <c r="I25" s="37" t="n"/>
-      <c r="J25" s="37" t="n"/>
-      <c r="K25" s="37" t="n"/>
-      <c r="L25" s="38" t="n"/>
-      <c r="M25" s="38" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="46" t="inlineStr">
-        <is>
-          <t>Note: Format follows SEEA EA Table 7.1 (supply and use of ecosystem services). Carbon sequestration use allocated to Global/Exports as the benefit accrues globally.</t>
-        </is>
+      <c r="B22" s="55" t="inlineStr">
+        <is>
+          <t>USD thousands</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="56" t="n"/>
+      <c r="J22" s="56" t="n"/>
+      <c r="K22" s="56" t="n"/>
+      <c r="L22" s="57">
+        <f>SUM(C22:H22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="54" t="inlineStr">
+        <is>
+          <t>Nursery habitat</t>
+        </is>
+      </c>
+      <c r="B23" s="55" t="inlineStr">
+        <is>
+          <t>hectares</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="56" t="n"/>
+      <c r="J23" s="56" t="n"/>
+      <c r="K23" s="56" t="n"/>
+      <c r="L23" s="57">
+        <f>SUM(C23:H23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="60" t="inlineStr">
+        <is>
+          <t>Cultural (SEEA EA 6.6)</t>
+        </is>
+      </c>
+      <c r="B24" s="50" t="n"/>
+      <c r="C24" s="50" t="n"/>
+      <c r="D24" s="50" t="n"/>
+      <c r="E24" s="50" t="n"/>
+      <c r="F24" s="50" t="n"/>
+      <c r="G24" s="50" t="n"/>
+      <c r="H24" s="50" t="n"/>
+      <c r="I24" s="50" t="n"/>
+      <c r="J24" s="50" t="n"/>
+      <c r="K24" s="50" t="n"/>
+      <c r="L24" s="51" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="54" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="B25" s="55" t="inlineStr">
+        <is>
+          <t>visitor-days</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="56" t="n"/>
+      <c r="J25" s="56" t="n"/>
+      <c r="K25" s="56" t="n"/>
+      <c r="L25" s="57">
+        <f>SUM(C25:H25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="54" t="inlineStr">
+        <is>
+          <t>Gleaning</t>
+        </is>
+      </c>
+      <c r="B26" s="55" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7" t="n"/>
+      <c r="I26" s="56" t="n"/>
+      <c r="J26" s="56" t="n"/>
+      <c r="K26" s="56" t="n"/>
+      <c r="L26" s="57">
+        <f>SUM(C26:H26)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A28:M28"/>
-    <mergeCell ref="A19:M19"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="C2:H2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A23:M23"/>
-    <mergeCell ref="A6:M6"/>
-    <mergeCell ref="A17:M17"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="A10:M10"/>
-    <mergeCell ref="C15:H15"/>
+  <mergeCells count="12">
+    <mergeCell ref="A20:L20"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A13:L13"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A17:L17"/>
+    <mergeCell ref="A18:L18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>